<commit_message>
Metodología en iteraciones y actualizar gráficos de test estadístico
</commit_message>
<xml_diff>
--- a/statistical_analysis/mann_w-u-test2.xlsx
+++ b/statistical_analysis/mann_w-u-test2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udeaeduco-my.sharepoint.com/personal/santiago_vargas5_udea_edu_co/Documents/Estudio/PAI/Codigo/Code_Quindio/statistical_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{E2EABD2C-6FD5-4CB6-9825-0D3634F18EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B92B359-EB04-4637-B070-20DF9772FA37}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{E2EABD2C-6FD5-4CB6-9825-0D3634F18EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0AB454FD-4F9C-484B-AD1A-6C1A01C59A0C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="22">
   <si>
     <t>Fecha</t>
   </si>
@@ -117,7 +117,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -127,6 +127,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -158,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -166,6 +172,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -192,10 +200,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -483,16 +487,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J241"/>
+  <dimension ref="A1:M241"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -517,8 +522,14 @@
       <c r="J1" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>45503</v>
       </c>
@@ -543,8 +554,14 @@
       <c r="J2" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2">
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45510</v>
       </c>
@@ -563,14 +580,20 @@
       <c r="F3">
         <v>16</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="J3" s="3">
         <v>-8</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45518</v>
       </c>
@@ -589,14 +612,20 @@
       <c r="F4">
         <v>16</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="5" t="s">
         <v>8</v>
       </c>
       <c r="J4" s="3">
         <v>-5</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L4" t="s">
+        <v>9</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45525</v>
       </c>
@@ -621,8 +650,14 @@
       <c r="J5" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L5" t="s">
+        <v>12</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45531</v>
       </c>
@@ -641,14 +676,20 @@
       <c r="F6">
         <v>8</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="5" t="s">
         <v>10</v>
       </c>
       <c r="J6" s="3">
         <v>-9</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="M6">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45532</v>
       </c>
@@ -667,14 +708,20 @@
       <c r="F7">
         <v>16</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="5" t="s">
         <v>19</v>
       </c>
       <c r="J7" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="M7">
+        <v>-9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45539</v>
       </c>
@@ -699,8 +746,14 @@
       <c r="J8" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L8" t="s">
+        <v>11</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45546</v>
       </c>
@@ -719,14 +772,20 @@
       <c r="F9">
         <v>17</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J9" s="3">
         <v>-3</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L9" t="s">
+        <v>13</v>
+      </c>
+      <c r="M9">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45552</v>
       </c>
@@ -745,14 +804,20 @@
       <c r="F10">
         <v>9</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="5" t="s">
         <v>20</v>
       </c>
       <c r="J10" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L10" t="s">
+        <v>14</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>45560</v>
       </c>
@@ -778,7 +843,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>45567</v>
       </c>
@@ -804,7 +869,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>45574</v>
       </c>
@@ -830,7 +895,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>45581</v>
       </c>
@@ -850,7 +915,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>45588</v>
       </c>
@@ -869,8 +934,14 @@
       <c r="F15">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>45595</v>
       </c>
@@ -889,8 +960,14 @@
       <c r="F16">
         <v>48</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I16" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J16" s="3">
+        <v>-9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>45602</v>
       </c>
@@ -909,8 +986,14 @@
       <c r="F17">
         <v>48</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I17" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J17" s="3">
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>45609</v>
       </c>
@@ -929,8 +1012,14 @@
       <c r="F18">
         <v>48</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J18" s="3">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>45616</v>
       </c>
@@ -949,8 +1038,14 @@
       <c r="F19">
         <v>48</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J19" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>45623</v>
       </c>
@@ -969,8 +1064,20 @@
       <c r="F20">
         <v>48</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J20" s="3">
+        <v>-3</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M20" s="3">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>45630</v>
       </c>
@@ -989,8 +1096,14 @@
       <c r="F21">
         <v>48</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>45503</v>
       </c>
@@ -1009,8 +1122,14 @@
       <c r="F22">
         <v>8</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I22" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J22" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>45510</v>
       </c>
@@ -1029,8 +1148,14 @@
       <c r="F23">
         <v>16</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I23" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J23" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>45518</v>
       </c>
@@ -1049,8 +1174,14 @@
       <c r="F24">
         <v>16</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J24" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>45525</v>
       </c>
@@ -1070,7 +1201,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>45531</v>
       </c>
@@ -1090,7 +1221,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>45532</v>
       </c>
@@ -1110,7 +1241,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>45539</v>
       </c>
@@ -1130,7 +1261,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>45546</v>
       </c>
@@ -1150,7 +1281,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>45552</v>
       </c>
@@ -1170,7 +1301,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>45560</v>
       </c>
@@ -1190,7 +1321,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>45567</v>
       </c>

</xml_diff>